<commit_message>
Update negative price analysis 2026-04
</commit_message>
<xml_diff>
--- a/outputs/NSW_negative_prices.xlsx
+++ b/outputs/NSW_negative_prices.xlsx
@@ -449,7 +449,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J83"/>
+  <dimension ref="A1:J84"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -3304,6 +3304,40 @@
         <v>0</v>
       </c>
     </row>
+    <row r="84">
+      <c r="A84" s="2" t="inlineStr">
+        <is>
+          <t>Mar 2026</t>
+        </is>
+      </c>
+      <c r="B84" s="3" t="n">
+        <v>13.51</v>
+      </c>
+      <c r="C84" s="3" t="n">
+        <v>0.27</v>
+      </c>
+      <c r="D84" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="E84" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="F84" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="G84" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="H84" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="I84" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="J84" s="3" t="n">
+        <v>0</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -3315,7 +3349,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J83"/>
+  <dimension ref="A1:J84"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -6170,8 +6204,42 @@
         <v>0</v>
       </c>
     </row>
+    <row r="84">
+      <c r="A84" s="2" t="inlineStr">
+        <is>
+          <t>Mar 2026</t>
+        </is>
+      </c>
+      <c r="B84" s="3" t="n">
+        <v>13.51</v>
+      </c>
+      <c r="C84" s="3" t="n">
+        <v>0.27</v>
+      </c>
+      <c r="D84" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="E84" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="F84" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="G84" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="H84" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="I84" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="J84" s="3" t="n">
+        <v>0</v>
+      </c>
+    </row>
   </sheetData>
-  <conditionalFormatting sqref="B2:B83">
+  <conditionalFormatting sqref="B2:B84">
     <cfRule type="colorScale" priority="1">
       <colorScale>
         <cfvo type="min"/>
@@ -6183,7 +6251,7 @@
       </colorScale>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="C2:C83">
+  <conditionalFormatting sqref="C2:C84">
     <cfRule type="colorScale" priority="2">
       <colorScale>
         <cfvo type="min"/>
@@ -6195,7 +6263,7 @@
       </colorScale>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="D2:D83">
+  <conditionalFormatting sqref="D2:D84">
     <cfRule type="colorScale" priority="3">
       <colorScale>
         <cfvo type="min"/>
@@ -6207,7 +6275,7 @@
       </colorScale>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="E2:E83">
+  <conditionalFormatting sqref="E2:E84">
     <cfRule type="colorScale" priority="4">
       <colorScale>
         <cfvo type="min"/>
@@ -6219,7 +6287,7 @@
       </colorScale>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="F2:F83">
+  <conditionalFormatting sqref="F2:F84">
     <cfRule type="colorScale" priority="5">
       <colorScale>
         <cfvo type="min"/>
@@ -6231,7 +6299,7 @@
       </colorScale>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="G2:G83">
+  <conditionalFormatting sqref="G2:G84">
     <cfRule type="colorScale" priority="6">
       <colorScale>
         <cfvo type="min"/>
@@ -6243,7 +6311,7 @@
       </colorScale>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="H2:H83">
+  <conditionalFormatting sqref="H2:H84">
     <cfRule type="colorScale" priority="7">
       <colorScale>
         <cfvo type="min"/>
@@ -6255,7 +6323,7 @@
       </colorScale>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="I2:I83">
+  <conditionalFormatting sqref="I2:I84">
     <cfRule type="colorScale" priority="8">
       <colorScale>
         <cfvo type="min"/>
@@ -6267,7 +6335,7 @@
       </colorScale>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="J2:J83">
+  <conditionalFormatting sqref="J2:J84">
     <cfRule type="colorScale" priority="9">
       <colorScale>
         <cfvo type="min"/>
@@ -6289,7 +6357,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K83"/>
+  <dimension ref="A1:K84"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -9396,6 +9464,43 @@
         <v>0</v>
       </c>
     </row>
+    <row r="84">
+      <c r="A84" s="5" t="inlineStr">
+        <is>
+          <t>Mar 2026</t>
+        </is>
+      </c>
+      <c r="B84" s="5" t="n">
+        <v>2976</v>
+      </c>
+      <c r="C84" s="6" t="n">
+        <v>402</v>
+      </c>
+      <c r="D84" s="6" t="n">
+        <v>8</v>
+      </c>
+      <c r="E84" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="F84" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="G84" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="H84" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="I84" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="J84" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="K84" s="6" t="n">
+        <v>0</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Update negative price analysis 2026-05
</commit_message>
<xml_diff>
--- a/outputs/NSW_negative_prices.xlsx
+++ b/outputs/NSW_negative_prices.xlsx
@@ -449,7 +449,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J84"/>
+  <dimension ref="A1:J85"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -3338,6 +3338,40 @@
         <v>0</v>
       </c>
     </row>
+    <row r="85">
+      <c r="A85" s="2" t="inlineStr">
+        <is>
+          <t>Apr 2026</t>
+        </is>
+      </c>
+      <c r="B85" s="3" t="n">
+        <v>19.2</v>
+      </c>
+      <c r="C85" s="3" t="n">
+        <v>2.15</v>
+      </c>
+      <c r="D85" s="3" t="n">
+        <v>0.49</v>
+      </c>
+      <c r="E85" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="F85" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="G85" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="H85" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="I85" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="J85" s="3" t="n">
+        <v>0</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -3349,7 +3383,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J84"/>
+  <dimension ref="A1:J85"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -6238,8 +6272,42 @@
         <v>0</v>
       </c>
     </row>
+    <row r="85">
+      <c r="A85" s="2" t="inlineStr">
+        <is>
+          <t>Apr 2026</t>
+        </is>
+      </c>
+      <c r="B85" s="3" t="n">
+        <v>19.2</v>
+      </c>
+      <c r="C85" s="3" t="n">
+        <v>2.15</v>
+      </c>
+      <c r="D85" s="3" t="n">
+        <v>0.49</v>
+      </c>
+      <c r="E85" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="F85" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="G85" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="H85" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="I85" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="J85" s="3" t="n">
+        <v>0</v>
+      </c>
+    </row>
   </sheetData>
-  <conditionalFormatting sqref="B2:B84">
+  <conditionalFormatting sqref="B2:B85">
     <cfRule type="colorScale" priority="1">
       <colorScale>
         <cfvo type="min"/>
@@ -6251,7 +6319,7 @@
       </colorScale>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="C2:C84">
+  <conditionalFormatting sqref="C2:C85">
     <cfRule type="colorScale" priority="2">
       <colorScale>
         <cfvo type="min"/>
@@ -6263,7 +6331,7 @@
       </colorScale>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="D2:D84">
+  <conditionalFormatting sqref="D2:D85">
     <cfRule type="colorScale" priority="3">
       <colorScale>
         <cfvo type="min"/>
@@ -6275,7 +6343,7 @@
       </colorScale>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="E2:E84">
+  <conditionalFormatting sqref="E2:E85">
     <cfRule type="colorScale" priority="4">
       <colorScale>
         <cfvo type="min"/>
@@ -6287,7 +6355,7 @@
       </colorScale>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="F2:F84">
+  <conditionalFormatting sqref="F2:F85">
     <cfRule type="colorScale" priority="5">
       <colorScale>
         <cfvo type="min"/>
@@ -6299,7 +6367,7 @@
       </colorScale>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="G2:G84">
+  <conditionalFormatting sqref="G2:G85">
     <cfRule type="colorScale" priority="6">
       <colorScale>
         <cfvo type="min"/>
@@ -6311,7 +6379,7 @@
       </colorScale>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="H2:H84">
+  <conditionalFormatting sqref="H2:H85">
     <cfRule type="colorScale" priority="7">
       <colorScale>
         <cfvo type="min"/>
@@ -6323,7 +6391,7 @@
       </colorScale>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="I2:I84">
+  <conditionalFormatting sqref="I2:I85">
     <cfRule type="colorScale" priority="8">
       <colorScale>
         <cfvo type="min"/>
@@ -6335,7 +6403,7 @@
       </colorScale>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="J2:J84">
+  <conditionalFormatting sqref="J2:J85">
     <cfRule type="colorScale" priority="9">
       <colorScale>
         <cfvo type="min"/>
@@ -6357,7 +6425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K84"/>
+  <dimension ref="A1:K85"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -9501,6 +9569,43 @@
         <v>0</v>
       </c>
     </row>
+    <row r="85">
+      <c r="A85" s="5" t="inlineStr">
+        <is>
+          <t>Apr 2026</t>
+        </is>
+      </c>
+      <c r="B85" s="5" t="n">
+        <v>2880</v>
+      </c>
+      <c r="C85" s="6" t="n">
+        <v>553</v>
+      </c>
+      <c r="D85" s="6" t="n">
+        <v>62</v>
+      </c>
+      <c r="E85" s="6" t="n">
+        <v>14</v>
+      </c>
+      <c r="F85" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="G85" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="H85" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="I85" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="J85" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="K85" s="6" t="n">
+        <v>0</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Update negative price analysis 2026-07
</commit_message>
<xml_diff>
--- a/outputs/NSW_negative_prices.xlsx
+++ b/outputs/NSW_negative_prices.xlsx
@@ -449,7 +449,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J85"/>
+  <dimension ref="A1:J87"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -3372,6 +3372,74 @@
         <v>0</v>
       </c>
     </row>
+    <row r="86">
+      <c r="A86" s="2" t="inlineStr">
+        <is>
+          <t>May 2026</t>
+        </is>
+      </c>
+      <c r="B86" s="3" t="n">
+        <v>4.3</v>
+      </c>
+      <c r="C86" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="D86" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="E86" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="F86" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="G86" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="H86" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="I86" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="J86" s="3" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="87">
+      <c r="A87" s="2" t="inlineStr">
+        <is>
+          <t>Jun 2026</t>
+        </is>
+      </c>
+      <c r="B87" s="3" t="n">
+        <v>1.08</v>
+      </c>
+      <c r="C87" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="D87" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="E87" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="F87" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="G87" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="H87" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="I87" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="J87" s="3" t="n">
+        <v>0</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -3383,7 +3451,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J85"/>
+  <dimension ref="A1:J87"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -6306,8 +6374,76 @@
         <v>0</v>
       </c>
     </row>
+    <row r="86">
+      <c r="A86" s="2" t="inlineStr">
+        <is>
+          <t>May 2026</t>
+        </is>
+      </c>
+      <c r="B86" s="3" t="n">
+        <v>4.3</v>
+      </c>
+      <c r="C86" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="D86" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="E86" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="F86" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="G86" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="H86" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="I86" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="J86" s="3" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="87">
+      <c r="A87" s="2" t="inlineStr">
+        <is>
+          <t>Jun 2026</t>
+        </is>
+      </c>
+      <c r="B87" s="3" t="n">
+        <v>1.08</v>
+      </c>
+      <c r="C87" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="D87" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="E87" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="F87" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="G87" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="H87" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="I87" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="J87" s="3" t="n">
+        <v>0</v>
+      </c>
+    </row>
   </sheetData>
-  <conditionalFormatting sqref="B2:B85">
+  <conditionalFormatting sqref="B2:B87">
     <cfRule type="colorScale" priority="1">
       <colorScale>
         <cfvo type="min"/>
@@ -6319,7 +6455,7 @@
       </colorScale>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="C2:C85">
+  <conditionalFormatting sqref="C2:C87">
     <cfRule type="colorScale" priority="2">
       <colorScale>
         <cfvo type="min"/>
@@ -6331,7 +6467,7 @@
       </colorScale>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="D2:D85">
+  <conditionalFormatting sqref="D2:D87">
     <cfRule type="colorScale" priority="3">
       <colorScale>
         <cfvo type="min"/>
@@ -6343,7 +6479,7 @@
       </colorScale>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="E2:E85">
+  <conditionalFormatting sqref="E2:E87">
     <cfRule type="colorScale" priority="4">
       <colorScale>
         <cfvo type="min"/>
@@ -6355,7 +6491,7 @@
       </colorScale>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="F2:F85">
+  <conditionalFormatting sqref="F2:F87">
     <cfRule type="colorScale" priority="5">
       <colorScale>
         <cfvo type="min"/>
@@ -6367,7 +6503,7 @@
       </colorScale>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="G2:G85">
+  <conditionalFormatting sqref="G2:G87">
     <cfRule type="colorScale" priority="6">
       <colorScale>
         <cfvo type="min"/>
@@ -6379,7 +6515,7 @@
       </colorScale>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="H2:H85">
+  <conditionalFormatting sqref="H2:H87">
     <cfRule type="colorScale" priority="7">
       <colorScale>
         <cfvo type="min"/>
@@ -6391,7 +6527,7 @@
       </colorScale>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="I2:I85">
+  <conditionalFormatting sqref="I2:I87">
     <cfRule type="colorScale" priority="8">
       <colorScale>
         <cfvo type="min"/>
@@ -6403,7 +6539,7 @@
       </colorScale>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="J2:J85">
+  <conditionalFormatting sqref="J2:J87">
     <cfRule type="colorScale" priority="9">
       <colorScale>
         <cfvo type="min"/>
@@ -6425,7 +6561,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K85"/>
+  <dimension ref="A1:K87"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -9606,6 +9742,80 @@
         <v>0</v>
       </c>
     </row>
+    <row r="86">
+      <c r="A86" s="5" t="inlineStr">
+        <is>
+          <t>May 2026</t>
+        </is>
+      </c>
+      <c r="B86" s="5" t="n">
+        <v>2976</v>
+      </c>
+      <c r="C86" s="6" t="n">
+        <v>128</v>
+      </c>
+      <c r="D86" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="E86" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="F86" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="G86" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="H86" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="I86" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="J86" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="K86" s="6" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="87">
+      <c r="A87" s="5" t="inlineStr">
+        <is>
+          <t>Jun 2026</t>
+        </is>
+      </c>
+      <c r="B87" s="5" t="n">
+        <v>2880</v>
+      </c>
+      <c r="C87" s="6" t="n">
+        <v>31</v>
+      </c>
+      <c r="D87" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="E87" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="F87" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="G87" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="H87" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="I87" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="J87" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="K87" s="6" t="n">
+        <v>0</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>